<commit_message>
feat: tudo ok j
</commit_message>
<xml_diff>
--- a/public/modelo_salario.xlsx
+++ b/public/modelo_salario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projetos\gestao-viagens-csiprc\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0062E251-F38A-448F-AE11-D341B02EBB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526C0710-C56A-4307-9107-F70B33E638DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm_Print_Area" localSheetId="0">Planilha1!$A$1:$H$25</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Planilha1!$A$1:$H$25</definedName>
+    <definedName name="_xlnm_Print_Area" localSheetId="0">Planilha1!$A$1:$H$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Planilha1!$A$1:$H$24</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>CONTROLE DE VIAGENS - DIÁRIAS PARA SEREM INCLUÍDAS NO SALÁRIO</t>
   </si>
@@ -71,16 +71,12 @@
   <si>
     <t>VALOR</t>
   </si>
-  <si>
-    <t xml:space="preserve">TOTAL GERAL = </t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="[$R$-416]\ #,##0.00;[Red]\-[$R$-416]\ #,##0.00"/>
+  <numFmts count="1">
     <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
@@ -142,7 +138,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -165,56 +161,15 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -241,20 +196,11 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -502,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.44140625" customWidth="1"/>
@@ -516,76 +462,76 @@
   <sheetData>
     <row r="1" spans="1:8" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="16"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
     </row>
     <row r="3" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
     </row>
     <row r="4" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
     </row>
     <row r="5" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
     </row>
     <row r="6" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="16"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
     </row>
     <row r="7" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="16"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
     </row>
     <row r="9" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -613,266 +559,240 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="4" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
+    <row r="10" spans="1:8" s="2" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="4">
         <v>1</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:8" s="4" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="6">
+      <c r="B10" s="6"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" spans="1:8" s="2" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
         <v>2</v>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="1:8" s="5" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="6">
+      <c r="B11" s="6"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" spans="1:8" s="3" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
         <v>3</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:8" s="5" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="6">
+      <c r="B12" s="6"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" spans="1:8" s="3" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
         <v>4</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="1:8" s="5" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="6">
+      <c r="B13" s="6"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" spans="1:8" s="3" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
         <v>5</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="1:8" s="10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="6">
+      <c r="B14" s="6"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" spans="1:8" s="8" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="4">
         <v>6</v>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="7"/>
-    </row>
-    <row r="16" spans="1:8" s="10" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="6">
+      <c r="B15" s="6"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="5"/>
+    </row>
+    <row r="16" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="4">
         <v>7</v>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="7"/>
-    </row>
-    <row r="17" spans="1:8" s="10" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="6">
+      <c r="B16" s="6"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="5"/>
+    </row>
+    <row r="17" spans="1:8" s="8" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="4">
         <v>8</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="7"/>
-    </row>
-    <row r="18" spans="1:8" s="12" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="6">
+      <c r="B17" s="6"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" spans="1:8" s="10" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4">
         <v>9</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:8" s="12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="6">
+      <c r="B18" s="6"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" spans="1:8" s="10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="4">
         <v>10</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="7"/>
-    </row>
-    <row r="20" spans="1:8" s="12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="6">
+      <c r="B19" s="6"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="20" spans="1:8" s="10" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="4">
         <v>11</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="7"/>
-    </row>
-    <row r="21" spans="1:8" s="13" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="6">
+      <c r="B20" s="6"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" spans="1:8" s="11" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="4">
         <v>12</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="7"/>
-    </row>
-    <row r="22" spans="1:8" s="13" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="6">
+      <c r="B21" s="6"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="5"/>
+    </row>
+    <row r="22" spans="1:8" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="4">
         <v>13</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="7"/>
-    </row>
-    <row r="23" spans="1:8" s="13" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="6">
+      <c r="B22" s="6"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" spans="1:8" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="4">
         <v>14</v>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="7"/>
-    </row>
-    <row r="24" spans="1:8" s="12" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="6">
+      <c r="B23" s="6"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="1:8" s="10" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="4">
         <v>15</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="7"/>
-    </row>
-    <row r="25" spans="1:8" s="3" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="20"/>
-      <c r="H25" s="2">
-        <f>SUM(H10:H24)</f>
-        <v>0</v>
-      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
     </row>
     <row r="26" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="21"/>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
     </row>
     <row r="27" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
+      <c r="A27" s="14"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
     </row>
     <row r="28" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="21"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
+      <c r="A28" s="14"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
     </row>
     <row r="29" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="21"/>
-      <c r="B29" s="21"/>
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="21"/>
-    </row>
-    <row r="30" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="21"/>
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-    </row>
-    <row r="31" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="21"/>
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2:H7"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A25:G25"/>
   </mergeCells>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="76" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix: Adicionada vírgula na importação do motor de exclusão
</commit_message>
<xml_diff>
--- a/public/modelo_salario.xlsx
+++ b/public/modelo_salario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projetos\gestao-viagens-csiprc\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526C0710-C56A-4307-9107-F70B33E638DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC111E58-D67F-4C11-BCFB-E348DADEB200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -112,7 +112,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -128,12 +128,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor rgb="FFC0C0C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFC0C0C0"/>
       </patternFill>
     </fill>
@@ -165,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -175,7 +169,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -190,16 +184,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -462,76 +453,76 @@
   <sheetData>
     <row r="1" spans="1:8" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
     </row>
     <row r="3" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="15"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="15"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="6" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
     </row>
     <row r="7" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
     </row>
     <row r="9" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -566,7 +557,7 @@
       <c r="B10" s="6"/>
       <c r="C10" s="4"/>
       <c r="D10" s="7"/>
-      <c r="E10" s="12"/>
+      <c r="E10" s="15"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="5"/>
@@ -578,7 +569,7 @@
       <c r="B11" s="6"/>
       <c r="C11" s="4"/>
       <c r="D11" s="7"/>
-      <c r="E11" s="12"/>
+      <c r="E11" s="15"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="5"/>
@@ -590,7 +581,7 @@
       <c r="B12" s="6"/>
       <c r="C12" s="4"/>
       <c r="D12" s="7"/>
-      <c r="E12" s="12"/>
+      <c r="E12" s="15"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="5"/>
@@ -698,7 +689,7 @@
       <c r="B21" s="6"/>
       <c r="C21" s="4"/>
       <c r="D21" s="7"/>
-      <c r="E21" s="13"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="9"/>
       <c r="G21" s="4"/>
       <c r="H21" s="5"/>
@@ -740,62 +731,62 @@
       <c r="H24" s="5"/>
     </row>
     <row r="25" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="14"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
+      <c r="A25" s="12"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
+      <c r="A26" s="12"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="14"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="14"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
     </row>
     <row r="29" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="14"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H7"/>
     <mergeCell ref="A8:H8"/>
   </mergeCells>
-  <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="76" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adiciona auto-logout por inatividade e roteamento logado p/ o painel no hero
</commit_message>
<xml_diff>
--- a/public/modelo_salario.xlsx
+++ b/public/modelo_salario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projetos\gestao-viagens-csiprc\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4A3C5DC-4474-4580-8342-5575878F6AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D5F66C-3CE1-4A6C-AD8A-C2A3F636757A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -238,10 +238,11 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -251,7 +252,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -344,23 +344,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>379365</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2054602</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>27460</xdr:rowOff>
+      <xdr:rowOff>53594</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1898039</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>161880</xdr:rowOff>
+      <xdr:colOff>1424250</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>39757</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagem 1">
+        <xdr:cNvPr id="9" name="Imagem 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{167FDAA8-E385-9981-678B-13679F5D32AA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{586208EC-8F19-8D9F-8C86-3255A0E2DFC6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -376,12 +376,22 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3379311" y="27460"/>
-          <a:ext cx="4738296" cy="1246528"/>
+          <a:off x="2293141" y="53594"/>
+          <a:ext cx="5353005" cy="1284876"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw blurRad="292100" dist="139700" dir="2700000" algn="tl" rotWithShape="0">
+            <a:srgbClr val="333333">
+              <a:alpha val="65000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -512,121 +522,121 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="14"/>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
+      <c r="A1" s="13"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
     </row>
     <row r="2" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="14"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="13"/>
     </row>
     <row r="3" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="14"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="13"/>
     </row>
     <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="14"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="13"/>
     </row>
     <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="14"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="13"/>
     </row>
     <row r="6" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="13"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="14"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="13"/>
     </row>
     <row r="7" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="19"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="14"/>
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="19"/>
     </row>
     <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="G9" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H9" s="15" t="s">
+      <c r="H9" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I9" s="15" t="s">
+      <c r="I9" s="14" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>